<commit_message>
corrected amplifier attachment logic for IDT files
</commit_message>
<xml_diff>
--- a/example_workflow/PhiKZ014_B2_IDT.xlsx
+++ b/example_workflow/PhiKZ014_B2_IDT.xlsx
@@ -445,7 +445,7 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>CCTCGTAAATCCTCATCAaaATAACCGCTTTAGAAAGAGTTTCCA</t>
+          <t>CCTCGTAAATCCTCATCAaaCTTCCAATAACTAATTTGGATTTCT</t>
         </is>
       </c>
     </row>
@@ -457,7 +457,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>CTTCCAATAACTAATTTGGATTTCTaaATCATCCAGTAAACCGCC</t>
+          <t>ATAACCGCTTTAGAAAGAGTTTCCAaaATCATCCAGTAAACCGCC</t>
         </is>
       </c>
     </row>
@@ -469,7 +469,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>CCTCGTAAATCCTCATCAaaCTTCAGGGTTCTCCATTGCTTCACG</t>
+          <t>CCTCGTAAATCCTCATCAaaGGAGTTCACCAATAGTTTTGGGTTG</t>
         </is>
       </c>
     </row>
@@ -481,7 +481,7 @@
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
-          <t>GGAGTTCACCAATAGTTTTGGGTTGaaATCATCCAGTAAACCGCC</t>
+          <t>CTTCAGGGTTCTCCATTGCTTCACGaaATCATCCAGTAAACCGCC</t>
         </is>
       </c>
     </row>
@@ -493,7 +493,7 @@
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>CCTCGTAAATCCTCATCAaaATCATCACTGATTTCACGCGAGCAT</t>
+          <t>CCTCGTAAATCCTCATCAaaCGAGTCGTCGTACATATCAAACACA</t>
         </is>
       </c>
     </row>
@@ -505,7 +505,7 @@
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>CGAGTCGTCGTACATATCAAACACAaaATCATCCAGTAAACCGCC</t>
+          <t>ATCATCACTGATTTCACGCGAGCATaaATCATCCAGTAAACCGCC</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
-          <t>CCTCGTAAATCCTCATCAaaAGATCATCATCATCCAGGGGCGTGC</t>
+          <t>CCTCGTAAATCCTCATCAaaTCATTCCATGAATAGCTTGATTCAT</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
-          <t>TCATTCCATGAATAGCTTGATTCATaaATCATCCAGTAAACCGCC</t>
+          <t>AGATCATCATCATCCAGGGGCGTGCaaATCATCCAGTAAACCGCC</t>
         </is>
       </c>
     </row>
@@ -541,7 +541,7 @@
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
-          <t>CCTCGTAAATCCTCATCAaaAGGTATCATCAGACTCACCATACTG</t>
+          <t>CCTCGTAAATCCTCATCAaaCACTGAGGTCACGGTCCAGTTCAGC</t>
         </is>
       </c>
     </row>
@@ -553,7 +553,7 @@
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
-          <t>CACTGAGGTCACGGTCCAGTTCAGCaaATCATCCAGTAAACCGCC</t>
+          <t>AGGTATCATCAGACTCACCATACTGaaATCATCCAGTAAACCGCC</t>
         </is>
       </c>
     </row>
@@ -565,7 +565,7 @@
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
-          <t>CCTCGTAAATCCTCATCAaaATACATCTCGCTAATTGCTTTATCG</t>
+          <t>CCTCGTAAATCCTCATCAaaTTCTTCTTGCGCCTTACGACGAGAA</t>
         </is>
       </c>
     </row>
@@ -577,7 +577,7 @@
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
-          <t>TTCTTCTTGCGCCTTACGACGAGAAaaATCATCCAGTAAACCGCC</t>
+          <t>ATACATCTCGCTAATTGCTTTATCGaaATCATCCAGTAAACCGCC</t>
         </is>
       </c>
     </row>
@@ -589,7 +589,7 @@
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
-          <t>CCTCGTAAATCCTCATCAaaTTGTAGAACGGAAGCAGGCGTTGCA</t>
+          <t>CCTCGTAAATCCTCATCAaaACTTTATGGAACTTCTTCTTGCTGA</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
-          <t>ACTTTATGGAACTTCTTCTTGCTGAaaATCATCCAGTAAACCGCC</t>
+          <t>TTGTAGAACGGAAGCAGGCGTTGCAaaATCATCCAGTAAACCGCC</t>
         </is>
       </c>
     </row>
@@ -613,7 +613,7 @@
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
-          <t>CCTCGTAAATCCTCATCAaaACCAGCTAACAGAGTAGCGAGACAG</t>
+          <t>CCTCGTAAATCCTCATCAaaTTACTTCAGCTGCTTTGATAGTCGG</t>
         </is>
       </c>
     </row>
@@ -625,7 +625,7 @@
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
-          <t>TTACTTCAGCTGCTTTGATAGTCGGaaATCATCCAGTAAACCGCC</t>
+          <t>ACCAGCTAACAGAGTAGCGAGACAGaaATCATCCAGTAAACCGCC</t>
         </is>
       </c>
     </row>
@@ -637,7 +637,7 @@
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
-          <t>CCTCGTAAATCCTCATCAaaGGAGTACAGCGCCATGACTAGCTTG</t>
+          <t>CCTCGTAAATCCTCATCAaaCAGTTTGTGCAGATGATCTTTAAAC</t>
         </is>
       </c>
     </row>
@@ -649,7 +649,7 @@
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
-          <t>CAGTTTGTGCAGATGATCTTTAAACaaATCATCCAGTAAACCGCC</t>
+          <t>GGAGTACAGCGCCATGACTAGCTTGaaATCATCCAGTAAACCGCC</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
-          <t>CCTCGTAAATCCTCATCAaaTTTGCATAAGCAGGATGTTCCCGAA</t>
+          <t>CCTCGTAAATCCTCATCAaaGTGAACATCACAAACGAACGCATGT</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
-          <t>GTGAACATCACAAACGAACGCATGTaaATCATCCAGTAAACCGCC</t>
+          <t>TTTGCATAAGCAGGATGTTCCCGAAaaATCATCCAGTAAACCGCC</t>
         </is>
       </c>
     </row>
@@ -685,7 +685,7 @@
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
-          <t>CCTCGTAAATCCTCATCAaaTGATATAGTACTGACTGTGATGTTT</t>
+          <t>CCTCGTAAATCCTCATCAaaTGATTTCGATGTATACCGGATCTAC</t>
         </is>
       </c>
     </row>
@@ -697,7 +697,7 @@
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
-          <t>TGATTTCGATGTATACCGGATCTACaaATCATCCAGTAAACCGCC</t>
+          <t>TGATATAGTACTGACTGTGATGTTTaaATCATCCAGTAAACCGCC</t>
         </is>
       </c>
     </row>
@@ -709,7 +709,7 @@
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
-          <t>CCTCGTAAATCCTCATCAaaGCGGTTATAATCGAATTCCTCTGCC</t>
+          <t>CCTCGTAAATCCTCATCAaaGGTAAGGCTACGTACTTTAGTAGGA</t>
         </is>
       </c>
     </row>
@@ -721,7 +721,7 @@
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
-          <t>GGTAAGGCTACGTACTTTAGTAGGAaaATCATCCAGTAAACCGCC</t>
+          <t>GCGGTTATAATCGAATTCCTCTGCCaaATCATCCAGTAAACCGCC</t>
         </is>
       </c>
     </row>
@@ -733,7 +733,7 @@
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
-          <t>CCTCGTAAATCCTCATCAaaGGACCTTCTGCCCAACGAACAGTCG</t>
+          <t>CCTCGTAAATCCTCATCAaaTGTTTCTCACGGATGTTCCAACCAT</t>
         </is>
       </c>
     </row>
@@ -745,7 +745,7 @@
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
-          <t>TGTTTCTCACGGATGTTCCAACCATaaATCATCCAGTAAACCGCC</t>
+          <t>GGACCTTCTGCCCAACGAACAGTCGaaATCATCCAGTAAACCGCC</t>
         </is>
       </c>
     </row>
@@ -757,7 +757,7 @@
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
-          <t>CCTCGTAAATCCTCATCAaaTGCGATCATACTCGGTTGACTCTTC</t>
+          <t>CCTCGTAAATCCTCATCAaaTGAACCAGGTGAAATTACCTTCACC</t>
         </is>
       </c>
     </row>
@@ -769,7 +769,7 @@
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
-          <t>TGAACCAGGTGAAATTACCTTCACCaaATCATCCAGTAAACCGCC</t>
+          <t>TGCGATCATACTCGGTTGACTCTTCaaATCATCCAGTAAACCGCC</t>
         </is>
       </c>
     </row>
@@ -781,7 +781,7 @@
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
-          <t>CCTCGTAAATCCTCATCAaaCGATACAATACCACGGCACCAACTG</t>
+          <t>CCTCGTAAATCCTCATCAaaGTTGATTGCCTTGTTACGGCTTTCA</t>
         </is>
       </c>
     </row>
@@ -793,7 +793,7 @@
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
-          <t>GTTGATTGCCTTGTTACGGCTTTCAaaATCATCCAGTAAACCGCC</t>
+          <t>CGATACAATACCACGGCACCAACTGaaATCATCCAGTAAACCGCC</t>
         </is>
       </c>
     </row>
@@ -805,7 +805,7 @@
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
-          <t>CCTCGTAAATCCTCATCAaaAGATCACAGGGCATGTCCAGAATAG</t>
+          <t>CCTCGTAAATCCTCATCAaaACATAACTGTTATGACCATTGGCCA</t>
         </is>
       </c>
     </row>
@@ -817,7 +817,7 @@
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
-          <t>ACATAACTGTTATGACCATTGGCCAaaATCATCCAGTAAACCGCC</t>
+          <t>AGATCACAGGGCATGTCCAGAATAGaaATCATCCAGTAAACCGCC</t>
         </is>
       </c>
     </row>
@@ -829,7 +829,7 @@
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
-          <t>CCTCGTAAATCCTCATCAaaCGCCGAGAACAGTAGCTTCGAATGT</t>
+          <t>CCTCGTAAATCCTCATCAaaCGTAGCGCTGTCCAGGATACACACG</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
-          <t>CGTAGCGCTGTCCAGGATACACACGaaATCATCCAGTAAACCGCC</t>
+          <t>CGCCGAGAACAGTAGCTTCGAATGTaaATCATCCAGTAAACCGCC</t>
         </is>
       </c>
     </row>
@@ -853,7 +853,7 @@
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
-          <t>CCTCGTAAATCCTCATCAaaATTCTCATCCAGGTAACGAAGGGAG</t>
+          <t>CCTCGTAAATCCTCATCAaaGGATTCGAAGATAGCACGAGTACCG</t>
         </is>
       </c>
     </row>
@@ -865,7 +865,7 @@
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
-          <t>GGATTCGAAGATAGCACGAGTACCGaaATCATCCAGTAAACCGCC</t>
+          <t>ATTCTCATCCAGGTAACGAAGGGAGaaATCATCCAGTAAACCGCC</t>
         </is>
       </c>
     </row>
@@ -877,7 +877,7 @@
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
-          <t>CCTCGTAAATCCTCATCAaaGGGAAATGGGCACGACCGAAAGGTT</t>
+          <t>CCTCGTAAATCCTCATCAaaTCGGCCTTTCTTTCTTTACGACGGC</t>
         </is>
       </c>
     </row>
@@ -889,7 +889,7 @@
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
-          <t>TCGGCCTTTCTTTCTTTACGACGGCaaATCATCCAGTAAACCGCC</t>
+          <t>GGGAAATGGGCACGACCGAAAGGTTaaATCATCCAGTAAACCGCC</t>
         </is>
       </c>
     </row>

</xml_diff>